<commit_message>
Added designators to BOM
</commit_message>
<xml_diff>
--- a/PCBs/ToF-Breakout-Board/BOM_ToF_board.xlsx
+++ b/PCBs/ToF-Breakout-Board/BOM_ToF_board.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shepl\OneDrive\Documents\7-MIL\TerraGator\ToF-Breakout-Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\russe\Repositories\MIL\TerraGator\PCBs\ToF-Breakout-Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84FD48B3-49D6-425C-A712-42E8ADF6BB11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D21A049E-FBBB-4CD0-959F-D654CBF45AB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2544" yWindow="2544" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="My Lists Worksheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="114">
   <si>
     <t>Country of Origin may be different at time of shipment.</t>
   </si>
@@ -341,6 +341,27 @@
   </si>
   <si>
     <t>https://mm.digikey.com/Volume0/opasdata/d220001/medias/images/2878/MFG_VL53L1CXV0FY%5E1.jpg</t>
+  </si>
+  <si>
+    <t>Designator</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>C1, C2</t>
+  </si>
+  <si>
+    <t>C3</t>
   </si>
 </sst>
 </file>
@@ -709,701 +730,727 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AF9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AG9"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="10.81640625" customWidth="1"/>
+    <col min="3" max="3" width="17.26953125" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>107</v>
+      </c>
+      <c r="C3" t="s">
         <v>3</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>4</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>5</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>6</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>7</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>8</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>9</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>10</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>11</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>12</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>13</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>14</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>15</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>16</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>17</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>18</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>19</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>20</v>
       </c>
-      <c r="T3" t="s">
+      <c r="U3" t="s">
         <v>21</v>
       </c>
-      <c r="U3" t="s">
+      <c r="V3" t="s">
         <v>22</v>
       </c>
-      <c r="V3" t="s">
+      <c r="W3" t="s">
         <v>23</v>
       </c>
-      <c r="W3" t="s">
+      <c r="X3" t="s">
         <v>24</v>
       </c>
-      <c r="X3" t="s">
+      <c r="Y3" t="s">
         <v>25</v>
       </c>
-      <c r="Y3" t="s">
+      <c r="Z3" t="s">
         <v>26</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" t="s">
         <v>27</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AB3" t="s">
         <v>28</v>
       </c>
-      <c r="AB3" t="s">
+      <c r="AC3" t="s">
         <v>29</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AD3" t="s">
         <v>30</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AE3" t="s">
         <v>31</v>
       </c>
-      <c r="AE3" t="s">
+      <c r="AF3" t="s">
         <v>32</v>
       </c>
-      <c r="AF3" t="s">
+      <c r="AG3" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C4" t="s">
         <v>34</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>35</v>
       </c>
-      <c r="D4" t="s">
+      <c r="E4" t="s">
         <v>36</v>
       </c>
-      <c r="E4" t="s">
-        <v>37</v>
-      </c>
       <c r="F4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" t="s">
         <v>38</v>
       </c>
-      <c r="G4" t="s">
+      <c r="H4" t="s">
         <v>39</v>
-      </c>
-      <c r="I4">
-        <v>7</v>
       </c>
       <c r="J4">
         <v>7</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4">
+        <v>7</v>
+      </c>
+      <c r="L4" t="s">
         <v>40</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>41</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>42</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>43</v>
       </c>
-      <c r="O4">
+      <c r="P4">
         <v>1</v>
       </c>
-      <c r="P4" t="s">
-        <v>37</v>
-      </c>
       <c r="Q4" t="s">
+        <v>37</v>
+      </c>
+      <c r="R4" t="s">
         <v>44</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>45</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>46</v>
       </c>
-      <c r="T4" t="s">
-        <v>37</v>
-      </c>
       <c r="U4" t="s">
+        <v>37</v>
+      </c>
+      <c r="V4" t="s">
         <v>47</v>
       </c>
-      <c r="V4" t="s">
-        <v>37</v>
-      </c>
       <c r="W4" t="s">
+        <v>37</v>
+      </c>
+      <c r="X4" t="s">
         <v>48</v>
       </c>
-      <c r="X4" t="s">
+      <c r="Y4" t="s">
         <v>49</v>
       </c>
-      <c r="Y4" t="s">
+      <c r="Z4" t="s">
         <v>50</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="AA4" t="s">
         <v>51</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AB4" t="s">
         <v>52</v>
       </c>
-      <c r="AB4" t="s">
+      <c r="AC4" t="s">
         <v>53</v>
       </c>
-      <c r="AC4" t="s">
+      <c r="AD4" t="s">
         <v>54</v>
       </c>
-      <c r="AD4" t="s">
+      <c r="AE4" t="s">
         <v>44</v>
       </c>
-      <c r="AE4" t="s">
+      <c r="AF4" t="s">
         <v>55</v>
       </c>
-      <c r="AF4" t="s">
+      <c r="AG4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" t="s">
         <v>56</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>57</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
         <v>58</v>
       </c>
-      <c r="E5" t="s">
-        <v>37</v>
-      </c>
       <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
         <v>59</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>39</v>
-      </c>
-      <c r="I5">
-        <v>10</v>
       </c>
       <c r="J5">
         <v>10</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5">
+        <v>10</v>
+      </c>
+      <c r="L5" t="s">
         <v>40</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>60</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>61</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>62</v>
       </c>
-      <c r="O5">
+      <c r="P5">
         <v>1</v>
       </c>
-      <c r="P5" t="s">
-        <v>37</v>
-      </c>
       <c r="Q5" t="s">
+        <v>37</v>
+      </c>
+      <c r="R5" t="s">
         <v>63</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>64</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>65</v>
       </c>
-      <c r="T5" t="s">
-        <v>37</v>
-      </c>
       <c r="U5" t="s">
+        <v>37</v>
+      </c>
+      <c r="V5" t="s">
         <v>66</v>
       </c>
-      <c r="V5" t="s">
-        <v>37</v>
-      </c>
       <c r="W5" t="s">
+        <v>37</v>
+      </c>
+      <c r="X5" t="s">
         <v>48</v>
       </c>
-      <c r="X5" t="s">
+      <c r="Y5" t="s">
         <v>49</v>
       </c>
-      <c r="Y5" t="s">
+      <c r="Z5" t="s">
         <v>67</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AA5" t="s">
         <v>51</v>
       </c>
-      <c r="AA5" t="s">
+      <c r="AB5" t="s">
         <v>68</v>
       </c>
-      <c r="AB5" t="s">
+      <c r="AC5" t="s">
         <v>69</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AD5" t="s">
         <v>70</v>
       </c>
-      <c r="AD5" t="s">
+      <c r="AE5" t="s">
         <v>63</v>
       </c>
-      <c r="AE5" t="s">
+      <c r="AF5" t="s">
         <v>71</v>
       </c>
-      <c r="AF5" t="s">
+      <c r="AG5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>3</v>
       </c>
       <c r="B6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6" t="s">
         <v>72</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>57</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>73</v>
       </c>
-      <c r="E6" t="s">
-        <v>37</v>
-      </c>
       <c r="F6" t="s">
+        <v>37</v>
+      </c>
+      <c r="G6" t="s">
         <v>74</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>39</v>
-      </c>
-      <c r="I6">
-        <v>10</v>
       </c>
       <c r="J6">
         <v>10</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6">
+        <v>10</v>
+      </c>
+      <c r="L6" t="s">
         <v>40</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>75</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>61</v>
       </c>
-      <c r="N6" t="s">
+      <c r="O6" t="s">
         <v>62</v>
       </c>
-      <c r="O6">
+      <c r="P6">
         <v>1</v>
       </c>
-      <c r="P6" t="s">
-        <v>37</v>
-      </c>
       <c r="Q6" t="s">
+        <v>37</v>
+      </c>
+      <c r="R6" t="s">
         <v>75</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>64</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>65</v>
       </c>
-      <c r="T6" t="s">
-        <v>37</v>
-      </c>
       <c r="U6" t="s">
+        <v>37</v>
+      </c>
+      <c r="V6" t="s">
         <v>66</v>
       </c>
-      <c r="V6" t="s">
-        <v>37</v>
-      </c>
       <c r="W6" t="s">
+        <v>37</v>
+      </c>
+      <c r="X6" t="s">
         <v>48</v>
       </c>
-      <c r="X6" t="s">
+      <c r="Y6" t="s">
         <v>49</v>
       </c>
-      <c r="Y6" t="s">
+      <c r="Z6" t="s">
         <v>67</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AA6" t="s">
         <v>51</v>
       </c>
-      <c r="AA6" t="s">
+      <c r="AB6" t="s">
         <v>68</v>
       </c>
-      <c r="AB6" t="s">
+      <c r="AC6" t="s">
         <v>69</v>
       </c>
-      <c r="AC6" t="s">
+      <c r="AD6" t="s">
         <v>70</v>
       </c>
-      <c r="AD6" t="s">
+      <c r="AE6" t="s">
         <v>75</v>
       </c>
-      <c r="AE6" t="s">
+      <c r="AF6" t="s">
         <v>71</v>
       </c>
-      <c r="AF6" t="s">
+      <c r="AG6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>4</v>
       </c>
       <c r="B7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" t="s">
         <v>76</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>77</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>78</v>
       </c>
-      <c r="E7" t="s">
-        <v>37</v>
-      </c>
       <c r="F7" t="s">
+        <v>37</v>
+      </c>
+      <c r="G7" t="s">
         <v>79</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>39</v>
-      </c>
-      <c r="I7">
-        <v>20</v>
       </c>
       <c r="J7">
         <v>20</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7">
+        <v>20</v>
+      </c>
+      <c r="L7" t="s">
         <v>40</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>80</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>81</v>
       </c>
-      <c r="N7" t="s">
+      <c r="O7" t="s">
         <v>82</v>
       </c>
-      <c r="O7">
+      <c r="P7">
         <v>1</v>
       </c>
-      <c r="P7" t="s">
-        <v>37</v>
-      </c>
       <c r="Q7" t="s">
+        <v>37</v>
+      </c>
+      <c r="R7" t="s">
         <v>80</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>83</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>84</v>
       </c>
-      <c r="T7" t="s">
-        <v>37</v>
-      </c>
       <c r="U7" t="s">
+        <v>37</v>
+      </c>
+      <c r="V7" t="s">
         <v>47</v>
       </c>
-      <c r="V7" t="s">
-        <v>37</v>
-      </c>
       <c r="W7" t="s">
+        <v>37</v>
+      </c>
+      <c r="X7" t="s">
         <v>48</v>
       </c>
-      <c r="X7" t="s">
+      <c r="Y7" t="s">
         <v>49</v>
       </c>
-      <c r="Y7" t="s">
+      <c r="Z7" t="s">
         <v>67</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="AA7" t="s">
         <v>51</v>
       </c>
-      <c r="AA7" t="s">
+      <c r="AB7" t="s">
         <v>85</v>
       </c>
-      <c r="AB7" t="s">
+      <c r="AC7" t="s">
         <v>53</v>
       </c>
-      <c r="AC7" t="s">
-        <v>37</v>
-      </c>
       <c r="AD7" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE7" t="s">
         <v>80</v>
       </c>
-      <c r="AE7" t="s">
+      <c r="AF7" t="s">
         <v>71</v>
       </c>
-      <c r="AF7" t="s">
+      <c r="AG7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>5</v>
       </c>
       <c r="B8" t="s">
+        <v>113</v>
+      </c>
+      <c r="C8" t="s">
         <v>86</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>87</v>
       </c>
-      <c r="D8" t="s">
+      <c r="E8" t="s">
         <v>88</v>
       </c>
-      <c r="E8" t="s">
-        <v>37</v>
-      </c>
       <c r="F8" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" t="s">
         <v>89</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>39</v>
-      </c>
-      <c r="I8">
-        <v>10</v>
       </c>
       <c r="J8">
         <v>10</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8">
+        <v>10</v>
+      </c>
+      <c r="L8" t="s">
         <v>40</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>90</v>
       </c>
-      <c r="M8" t="s">
+      <c r="N8" t="s">
         <v>91</v>
       </c>
-      <c r="N8" t="s">
+      <c r="O8" t="s">
         <v>92</v>
       </c>
-      <c r="O8">
+      <c r="P8">
         <v>1</v>
       </c>
-      <c r="P8" t="s">
-        <v>37</v>
-      </c>
       <c r="Q8" t="s">
+        <v>37</v>
+      </c>
+      <c r="R8" t="s">
         <v>90</v>
       </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>93</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>94</v>
       </c>
-      <c r="T8" t="s">
-        <v>37</v>
-      </c>
       <c r="U8" t="s">
+        <v>37</v>
+      </c>
+      <c r="V8" t="s">
         <v>66</v>
       </c>
-      <c r="V8" t="s">
-        <v>37</v>
-      </c>
       <c r="W8" t="s">
+        <v>37</v>
+      </c>
+      <c r="X8" t="s">
         <v>48</v>
       </c>
-      <c r="X8" t="s">
+      <c r="Y8" t="s">
         <v>49</v>
       </c>
-      <c r="Y8" t="s">
+      <c r="Z8" t="s">
         <v>67</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="AA8" t="s">
         <v>51</v>
       </c>
-      <c r="AA8" t="s">
+      <c r="AB8" t="s">
         <v>85</v>
       </c>
-      <c r="AB8" t="s">
+      <c r="AC8" t="s">
         <v>95</v>
       </c>
-      <c r="AC8" t="s">
-        <v>37</v>
-      </c>
       <c r="AD8" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE8" t="s">
         <v>90</v>
       </c>
-      <c r="AE8" t="s">
+      <c r="AF8" t="s">
         <v>71</v>
       </c>
-      <c r="AF8" t="s">
+      <c r="AG8" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>6</v>
       </c>
       <c r="B9" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" t="s">
         <v>96</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>97</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>98</v>
       </c>
-      <c r="E9" t="s">
-        <v>37</v>
-      </c>
       <c r="F9" t="s">
+        <v>37</v>
+      </c>
+      <c r="G9" t="s">
         <v>99</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>39</v>
-      </c>
-      <c r="I9">
-        <v>7</v>
       </c>
       <c r="J9">
         <v>7</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9">
+        <v>7</v>
+      </c>
+      <c r="L9" t="s">
         <v>40</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>100</v>
       </c>
-      <c r="M9" t="s">
+      <c r="N9" t="s">
         <v>101</v>
       </c>
-      <c r="N9" t="s">
+      <c r="O9" t="s">
         <v>102</v>
       </c>
-      <c r="O9">
+      <c r="P9">
         <v>1</v>
       </c>
-      <c r="P9" t="s">
-        <v>37</v>
-      </c>
       <c r="Q9" t="s">
+        <v>37</v>
+      </c>
+      <c r="R9" t="s">
         <v>100</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>103</v>
       </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>104</v>
       </c>
-      <c r="T9" t="s">
-        <v>37</v>
-      </c>
       <c r="U9" t="s">
+        <v>37</v>
+      </c>
+      <c r="V9" t="s">
         <v>47</v>
       </c>
-      <c r="V9" t="s">
-        <v>37</v>
-      </c>
       <c r="W9" t="s">
+        <v>37</v>
+      </c>
+      <c r="X9" t="s">
         <v>48</v>
       </c>
-      <c r="X9" t="s">
+      <c r="Y9" t="s">
         <v>49</v>
       </c>
-      <c r="Y9" t="s">
+      <c r="Z9" t="s">
         <v>50</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="AA9" t="s">
         <v>51</v>
       </c>
-      <c r="AA9" t="s">
+      <c r="AB9" t="s">
         <v>105</v>
       </c>
-      <c r="AB9" t="s">
+      <c r="AC9" t="s">
         <v>53</v>
       </c>
-      <c r="AC9" t="s">
-        <v>37</v>
-      </c>
       <c r="AD9" t="s">
+        <v>37</v>
+      </c>
+      <c r="AE9" t="s">
         <v>100</v>
       </c>
-      <c r="AE9" t="s">
+      <c r="AF9" t="s">
         <v>106</v>
       </c>
-      <c r="AF9" t="s">
+      <c r="AG9" t="s">
         <v>37</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="S4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="AE4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="S5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="AE5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="S6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="AE6" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="S7" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="AE7" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="S8" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="AE8" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="S9" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="AE9" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="T4" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="AF4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="T5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="AF5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="T6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="AF6" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="T7" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="AF7" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="T8" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="AF8" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="T9" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="AF9" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>